<commit_message>
Corrected Chile Database error for parsing in two rows
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/SVZ_Chile_Table1_merged.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/SVZ_Chile_Table1_merged.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\Gesammelte_Datenbanken\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94a36cc37384f3e2/SPEICHER/Hochschule/7. Semester/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96DE58AE-BFDA-41C9-BFB4-64B5D970D254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{96DE58AE-BFDA-41C9-BFB4-64B5D970D254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24EB70F2-DE2D-480A-B1D6-276A41E20E04}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TABLE1" sheetId="1" r:id="rId1"/>
@@ -1012,15 +1012,18 @@
         <v>881.79</v>
       </c>
       <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
         <v>58.1</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>26.6</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>81.3</v>
       </c>
-      <c r="Q4">
+      <c r="R4">
         <v>52</v>
       </c>
       <c r="S4">
@@ -1181,15 +1184,18 @@
         <v>2258</v>
       </c>
       <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
         <v>22.9</v>
       </c>
-      <c r="O6">
+      <c r="P6">
         <v>12.5</v>
       </c>
-      <c r="P6">
+      <c r="Q6">
         <v>35.5</v>
       </c>
-      <c r="Q6">
+      <c r="R6">
         <v>24.2</v>
       </c>
       <c r="S6">
@@ -1258,15 +1264,18 @@
         <v>414.52</v>
       </c>
       <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
         <v>27.7</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>12.4</v>
       </c>
-      <c r="P7">
+      <c r="Q7">
         <v>20.9</v>
       </c>
-      <c r="Q7">
+      <c r="R7">
         <v>2.4</v>
       </c>
       <c r="S7">

</xml_diff>